<commit_message>
Update: changed wikidata field names, tested new get_linked_entity function
</commit_message>
<xml_diff>
--- a/inferences/jesuita-entrada_totals.xlsx
+++ b/inferences/jesuita-entrada_totals.xlsx
@@ -477,7 +477,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -517,7 +517,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>

</xml_diff>